<commit_message>
Poprawiony zepsuty excel TerytPoprawki
</commit_message>
<xml_diff>
--- a/TerytLoad/AppData/pna/BledyPnaPropozycje.xlsx
+++ b/TerytLoad/AppData/pna/BledyPnaPropozycje.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Błędy PNA" sheetId="1" r:id="R0353f86735be40b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Błędy PNA" sheetId="1" r:id="R22ecf8e8e44e49dc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -55,17 +55,17 @@
     <x:row r="2">
       <x:c r="A2" t="inlineStr">
         <x:is>
-          <x:t>58-506</x:t>
+          <x:t>15-257</x:t>
         </x:is>
       </x:c>
       <x:c r="B2" t="inlineStr">
         <x:is>
-          <x:t>Jelenia Góra</x:t>
+          <x:t>Białystok</x:t>
         </x:is>
       </x:c>
       <x:c r="C2" t="inlineStr">
         <x:is>
-          <x:t>Plac św. apostoła Jana</x:t>
+          <x:t>płk. Czesława Hake</x:t>
         </x:is>
       </x:c>
       <x:c r="D2" t="inlineStr">
@@ -75,17 +75,17 @@
       </x:c>
       <x:c r="E2" t="inlineStr">
         <x:is>
-          <x:t>Jelenia Góra</x:t>
+          <x:t>Białystok</x:t>
         </x:is>
       </x:c>
       <x:c r="F2" t="inlineStr">
         <x:is>
-          <x:t>Jelenia Góra</x:t>
+          <x:t>Białystok</x:t>
         </x:is>
       </x:c>
       <x:c r="G2" t="inlineStr">
         <x:is>
-          <x:t>dolnośląskie</x:t>
+          <x:t>podlaskie</x:t>
         </x:is>
       </x:c>
       <x:c r="H2" t="inlineStr">
@@ -97,17 +97,17 @@
     <x:row r="3">
       <x:c r="A3" t="inlineStr">
         <x:is>
-          <x:t>58-506</x:t>
+          <x:t>15-257</x:t>
         </x:is>
       </x:c>
       <x:c r="B3" t="inlineStr">
         <x:is>
-          <x:t>Jelenia Góra</x:t>
+          <x:t>Białystok</x:t>
         </x:is>
       </x:c>
       <x:c r="C3" t="inlineStr">
         <x:is>
-          <x:t>Plac św. apostoła Jana</x:t>
+          <x:t>płk. Czesława Hake</x:t>
         </x:is>
       </x:c>
       <x:c r="D3" t="inlineStr">
@@ -117,17 +117,17 @@
       </x:c>
       <x:c r="E3" t="inlineStr">
         <x:is>
-          <x:t>Jelenia Góra</x:t>
+          <x:t>Białystok</x:t>
         </x:is>
       </x:c>
       <x:c r="F3" t="inlineStr">
         <x:is>
-          <x:t>Jelenia Góra</x:t>
+          <x:t>Białystok</x:t>
         </x:is>
       </x:c>
       <x:c r="G3" t="inlineStr">
         <x:is>
-          <x:t>dolnośląskie</x:t>
+          <x:t>podlaskie</x:t>
         </x:is>
       </x:c>
       <x:c r="H3" t="inlineStr">
@@ -139,17 +139,17 @@
     <x:row r="4">
       <x:c r="A4" t="inlineStr">
         <x:is>
-          <x:t>30-198</x:t>
+          <x:t>80-834</x:t>
         </x:is>
       </x:c>
       <x:c r="B4" t="inlineStr">
         <x:is>
-          <x:t>Kraków</x:t>
+          <x:t>Gdańsk</x:t>
         </x:is>
       </x:c>
       <x:c r="C4" t="inlineStr">
         <x:is>
-          <x:t>mjr Łupaszki</x:t>
+          <x:t>św. Ducha</x:t>
         </x:is>
       </x:c>
       <x:c r="D4" t="inlineStr">
@@ -159,17 +159,17 @@
       </x:c>
       <x:c r="E4" t="inlineStr">
         <x:is>
-          <x:t>Kraków</x:t>
+          <x:t>Gdańsk</x:t>
         </x:is>
       </x:c>
       <x:c r="F4" t="inlineStr">
         <x:is>
-          <x:t>Kraków</x:t>
+          <x:t>Gdańsk</x:t>
         </x:is>
       </x:c>
       <x:c r="G4" t="inlineStr">
         <x:is>
-          <x:t>małopolskie</x:t>
+          <x:t>pomorskie</x:t>
         </x:is>
       </x:c>
       <x:c r="H4" t="inlineStr">
@@ -181,17 +181,17 @@
     <x:row r="5">
       <x:c r="A5" t="inlineStr">
         <x:is>
-          <x:t>30-198</x:t>
+          <x:t>80-834</x:t>
         </x:is>
       </x:c>
       <x:c r="B5" t="inlineStr">
         <x:is>
-          <x:t>Kraków</x:t>
+          <x:t>Gdańsk</x:t>
         </x:is>
       </x:c>
       <x:c r="C5" t="inlineStr">
         <x:is>
-          <x:t>mjr Łupaszki</x:t>
+          <x:t>św. Ducha</x:t>
         </x:is>
       </x:c>
       <x:c r="D5" t="inlineStr">
@@ -201,17 +201,17 @@
       </x:c>
       <x:c r="E5" t="inlineStr">
         <x:is>
-          <x:t>Kraków</x:t>
+          <x:t>Gdańsk</x:t>
         </x:is>
       </x:c>
       <x:c r="F5" t="inlineStr">
         <x:is>
-          <x:t>Kraków</x:t>
+          <x:t>Gdańsk</x:t>
         </x:is>
       </x:c>
       <x:c r="G5" t="inlineStr">
         <x:is>
-          <x:t>małopolskie</x:t>
+          <x:t>pomorskie</x:t>
         </x:is>
       </x:c>
       <x:c r="H5" t="inlineStr">
@@ -223,17 +223,17 @@
     <x:row r="6">
       <x:c r="A6" t="inlineStr">
         <x:is>
-          <x:t>48-300</x:t>
+          <x:t>81-577</x:t>
         </x:is>
       </x:c>
       <x:c r="B6" t="inlineStr">
         <x:is>
-          <x:t>Nysa</x:t>
+          <x:t>Gdynia</x:t>
         </x:is>
       </x:c>
       <x:c r="C6" t="inlineStr">
         <x:is>
-          <x:t>Generała Augusta Emila Fieldorfa-Pseudonim Nil</x:t>
+          <x:t>o. Pio</x:t>
         </x:is>
       </x:c>
       <x:c r="D6" t="inlineStr">
@@ -243,17 +243,17 @@
       </x:c>
       <x:c r="E6" t="inlineStr">
         <x:is>
-          <x:t>Nysa</x:t>
+          <x:t>Gdynia</x:t>
         </x:is>
       </x:c>
       <x:c r="F6" t="inlineStr">
         <x:is>
-          <x:t>nyski</x:t>
+          <x:t>Gdynia</x:t>
         </x:is>
       </x:c>
       <x:c r="G6" t="inlineStr">
         <x:is>
-          <x:t>opolskie</x:t>
+          <x:t>pomorskie</x:t>
         </x:is>
       </x:c>
       <x:c r="H6" t="inlineStr">
@@ -265,17 +265,17 @@
     <x:row r="7">
       <x:c r="A7" t="inlineStr">
         <x:is>
-          <x:t>48-300</x:t>
+          <x:t>81-577</x:t>
         </x:is>
       </x:c>
       <x:c r="B7" t="inlineStr">
         <x:is>
-          <x:t>Nysa</x:t>
+          <x:t>Gdynia</x:t>
         </x:is>
       </x:c>
       <x:c r="C7" t="inlineStr">
         <x:is>
-          <x:t>Generała Augusta Emila Fieldorfa-Pseudonim Nil</x:t>
+          <x:t>o. Pio</x:t>
         </x:is>
       </x:c>
       <x:c r="D7" t="inlineStr">
@@ -285,17 +285,17 @@
       </x:c>
       <x:c r="E7" t="inlineStr">
         <x:is>
-          <x:t>Nysa</x:t>
+          <x:t>Gdynia</x:t>
         </x:is>
       </x:c>
       <x:c r="F7" t="inlineStr">
         <x:is>
-          <x:t>nyski</x:t>
+          <x:t>Gdynia</x:t>
         </x:is>
       </x:c>
       <x:c r="G7" t="inlineStr">
         <x:is>
-          <x:t>opolskie</x:t>
+          <x:t>pomorskie</x:t>
         </x:is>
       </x:c>
       <x:c r="H7" t="inlineStr">
@@ -307,17 +307,17 @@
     <x:row r="8">
       <x:c r="A8" t="inlineStr">
         <x:is>
-          <x:t>71-602</x:t>
+          <x:t>58-506</x:t>
         </x:is>
       </x:c>
       <x:c r="B8" t="inlineStr">
         <x:is>
-          <x:t>Szczecin</x:t>
+          <x:t>Jelenia Góra</x:t>
         </x:is>
       </x:c>
       <x:c r="C8" t="inlineStr">
         <x:is>
-          <x:t>Storrady-Świętosławy</x:t>
+          <x:t>Plac św. apostoła Jana</x:t>
         </x:is>
       </x:c>
       <x:c r="D8" t="inlineStr">
@@ -327,17 +327,17 @@
       </x:c>
       <x:c r="E8" t="inlineStr">
         <x:is>
-          <x:t>Szczecin</x:t>
+          <x:t>Jelenia Góra</x:t>
         </x:is>
       </x:c>
       <x:c r="F8" t="inlineStr">
         <x:is>
-          <x:t>Szczecin</x:t>
+          <x:t>Jelenia Góra</x:t>
         </x:is>
       </x:c>
       <x:c r="G8" t="inlineStr">
         <x:is>
-          <x:t>zachodniopomorskie</x:t>
+          <x:t>dolnośląskie</x:t>
         </x:is>
       </x:c>
       <x:c r="H8" t="inlineStr">
@@ -349,17 +349,17 @@
     <x:row r="9">
       <x:c r="A9" t="inlineStr">
         <x:is>
-          <x:t>71-602</x:t>
+          <x:t>58-506</x:t>
         </x:is>
       </x:c>
       <x:c r="B9" t="inlineStr">
         <x:is>
-          <x:t>Szczecin</x:t>
+          <x:t>Jelenia Góra</x:t>
         </x:is>
       </x:c>
       <x:c r="C9" t="inlineStr">
         <x:is>
-          <x:t>Storrady-Świętosławy</x:t>
+          <x:t>Plac św. apostoła Jana</x:t>
         </x:is>
       </x:c>
       <x:c r="D9" t="inlineStr">
@@ -369,17 +369,17 @@
       </x:c>
       <x:c r="E9" t="inlineStr">
         <x:is>
-          <x:t>Szczecin</x:t>
+          <x:t>Jelenia Góra</x:t>
         </x:is>
       </x:c>
       <x:c r="F9" t="inlineStr">
         <x:is>
-          <x:t>Szczecin</x:t>
+          <x:t>Jelenia Góra</x:t>
         </x:is>
       </x:c>
       <x:c r="G9" t="inlineStr">
         <x:is>
-          <x:t>zachodniopomorskie</x:t>
+          <x:t>dolnośląskie</x:t>
         </x:is>
       </x:c>
       <x:c r="H9" t="inlineStr">
@@ -391,17 +391,17 @@
     <x:row r="10">
       <x:c r="A10" t="inlineStr">
         <x:is>
-          <x:t>43-100</x:t>
+          <x:t>46-200</x:t>
         </x:is>
       </x:c>
       <x:c r="B10" t="inlineStr">
         <x:is>
-          <x:t>Tychy</x:t>
+          <x:t>Kluczbork</x:t>
         </x:is>
       </x:c>
       <x:c r="C10" t="inlineStr">
         <x:is>
-          <x:t>van Beethovena</x:t>
+          <x:t>Generała Bema</x:t>
         </x:is>
       </x:c>
       <x:c r="D10" t="inlineStr">
@@ -411,17 +411,17 @@
       </x:c>
       <x:c r="E10" t="inlineStr">
         <x:is>
-          <x:t>Tychy</x:t>
+          <x:t>Kluczbork</x:t>
         </x:is>
       </x:c>
       <x:c r="F10" t="inlineStr">
         <x:is>
-          <x:t>Tychy</x:t>
+          <x:t>kluczborski</x:t>
         </x:is>
       </x:c>
       <x:c r="G10" t="inlineStr">
         <x:is>
-          <x:t>śląskie</x:t>
+          <x:t>opolskie</x:t>
         </x:is>
       </x:c>
       <x:c r="H10" t="inlineStr">
@@ -433,17 +433,17 @@
     <x:row r="11">
       <x:c r="A11" t="inlineStr">
         <x:is>
-          <x:t>43-100</x:t>
+          <x:t>46-200</x:t>
         </x:is>
       </x:c>
       <x:c r="B11" t="inlineStr">
         <x:is>
-          <x:t>Tychy</x:t>
+          <x:t>Kluczbork</x:t>
         </x:is>
       </x:c>
       <x:c r="C11" t="inlineStr">
         <x:is>
-          <x:t>van Beethovena</x:t>
+          <x:t>Generała Bema</x:t>
         </x:is>
       </x:c>
       <x:c r="D11" t="inlineStr">
@@ -453,17 +453,17 @@
       </x:c>
       <x:c r="E11" t="inlineStr">
         <x:is>
-          <x:t>Tychy</x:t>
+          <x:t>Kluczbork</x:t>
         </x:is>
       </x:c>
       <x:c r="F11" t="inlineStr">
         <x:is>
-          <x:t>Tychy</x:t>
+          <x:t>kluczborski</x:t>
         </x:is>
       </x:c>
       <x:c r="G11" t="inlineStr">
         <x:is>
-          <x:t>śląskie</x:t>
+          <x:t>opolskie</x:t>
         </x:is>
       </x:c>
       <x:c r="H11" t="inlineStr">
@@ -475,17 +475,17 @@
     <x:row r="12">
       <x:c r="A12" t="inlineStr">
         <x:is>
-          <x:t>66-006</x:t>
+          <x:t>91-492</x:t>
         </x:is>
       </x:c>
       <x:c r="B12" t="inlineStr">
         <x:is>
-          <x:t>Zielona Góra</x:t>
+          <x:t>Łódź</x:t>
         </x:is>
       </x:c>
       <x:c r="C12" t="inlineStr">
         <x:is>
-          <x:t>Ochla-Osiedle Dworskie</x:t>
+          <x:t>Generała Bema</x:t>
         </x:is>
       </x:c>
       <x:c r="D12" t="inlineStr">
@@ -495,17 +495,17 @@
       </x:c>
       <x:c r="E12" t="inlineStr">
         <x:is>
-          <x:t>Zielona Góra</x:t>
+          <x:t>Łódź</x:t>
         </x:is>
       </x:c>
       <x:c r="F12" t="inlineStr">
         <x:is>
-          <x:t>Zielona Góra</x:t>
+          <x:t>Łódź</x:t>
         </x:is>
       </x:c>
       <x:c r="G12" t="inlineStr">
         <x:is>
-          <x:t>lubuskie</x:t>
+          <x:t>łódzkie</x:t>
         </x:is>
       </x:c>
       <x:c r="H12" t="inlineStr">
@@ -517,40 +517,712 @@
     <x:row r="13">
       <x:c r="A13" t="inlineStr">
         <x:is>
+          <x:t>91-492</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B13" t="inlineStr">
+        <x:is>
+          <x:t>Łódź</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C13" t="inlineStr">
+        <x:is>
+          <x:t>Generała Bema</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D13" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E13" t="inlineStr">
+        <x:is>
+          <x:t>Łódź</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F13" t="inlineStr">
+        <x:is>
+          <x:t>Łódź</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G13" t="inlineStr">
+        <x:is>
+          <x:t>łódzkie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H13" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="inlineStr">
+        <x:is>
+          <x:t>48-300</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B14" t="inlineStr">
+        <x:is>
+          <x:t>Nysa</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C14" t="inlineStr">
+        <x:is>
+          <x:t>Generała Augusta Emila Fieldorfa-Pseudonim Nil</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D14" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E14" t="inlineStr">
+        <x:is>
+          <x:t>Nysa</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F14" t="inlineStr">
+        <x:is>
+          <x:t>nyski</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G14" t="inlineStr">
+        <x:is>
+          <x:t>opolskie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H14" t="inlineStr">
+        <x:is>
+          <x:t>Brak ulicy</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="inlineStr">
+        <x:is>
+          <x:t>48-300</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B15" t="inlineStr">
+        <x:is>
+          <x:t>Nysa</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C15" t="inlineStr">
+        <x:is>
+          <x:t>Generała Augusta Emila Fieldorfa-Pseudonim Nil</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D15" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E15" t="inlineStr">
+        <x:is>
+          <x:t>Nysa</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F15" t="inlineStr">
+        <x:is>
+          <x:t>nyski</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G15" t="inlineStr">
+        <x:is>
+          <x:t>opolskie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H15" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="inlineStr">
+        <x:is>
+          <x:t>42-256</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B16" t="inlineStr">
+        <x:is>
+          <x:t>Olsztyn</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C16" t="inlineStr">
+        <x:is>
+          <x:t>Plac im. marszałka Józefa Piłsudskiego</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D16" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E16" t="inlineStr">
+        <x:is>
+          <x:t>Olsztyn</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F16" t="inlineStr">
+        <x:is>
+          <x:t>częstochowski</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G16" t="inlineStr">
+        <x:is>
+          <x:t>śląskie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H16" t="inlineStr">
+        <x:is>
+          <x:t>Brak ulicy</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="inlineStr">
+        <x:is>
+          <x:t>42-256</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B17" t="inlineStr">
+        <x:is>
+          <x:t>Olsztyn</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C17" t="inlineStr">
+        <x:is>
+          <x:t>Plac im. marszałka Józefa Piłsudskiego</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D17" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E17" t="inlineStr">
+        <x:is>
+          <x:t>Olsztyn</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F17" t="inlineStr">
+        <x:is>
+          <x:t>częstochowski</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G17" t="inlineStr">
+        <x:is>
+          <x:t>śląskie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H17" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="inlineStr">
+        <x:is>
+          <x:t>71-602</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B18" t="inlineStr">
+        <x:is>
+          <x:t>Szczecin</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C18" t="inlineStr">
+        <x:is>
+          <x:t>Storrady-Świętosławy</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D18" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E18" t="inlineStr">
+        <x:is>
+          <x:t>Szczecin</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F18" t="inlineStr">
+        <x:is>
+          <x:t>Szczecin</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G18" t="inlineStr">
+        <x:is>
+          <x:t>zachodniopomorskie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H18" t="inlineStr">
+        <x:is>
+          <x:t>Brak ulicy</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="inlineStr">
+        <x:is>
+          <x:t>71-602</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B19" t="inlineStr">
+        <x:is>
+          <x:t>Szczecin</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C19" t="inlineStr">
+        <x:is>
+          <x:t>Storrady-Świętosławy</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D19" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E19" t="inlineStr">
+        <x:is>
+          <x:t>Szczecin</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F19" t="inlineStr">
+        <x:is>
+          <x:t>Szczecin</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G19" t="inlineStr">
+        <x:is>
+          <x:t>zachodniopomorskie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H19" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="inlineStr">
+        <x:is>
+          <x:t>43-100</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B20" t="inlineStr">
+        <x:is>
+          <x:t>Tychy</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C20" t="inlineStr">
+        <x:is>
+          <x:t>van Beethovena</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D20" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E20" t="inlineStr">
+        <x:is>
+          <x:t>Tychy</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F20" t="inlineStr">
+        <x:is>
+          <x:t>Tychy</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G20" t="inlineStr">
+        <x:is>
+          <x:t>śląskie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H20" t="inlineStr">
+        <x:is>
+          <x:t>Brak ulicy</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="inlineStr">
+        <x:is>
+          <x:t>43-100</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B21" t="inlineStr">
+        <x:is>
+          <x:t>Tychy</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C21" t="inlineStr">
+        <x:is>
+          <x:t>van Beethovena</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D21" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E21" t="inlineStr">
+        <x:is>
+          <x:t>Tychy</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F21" t="inlineStr">
+        <x:is>
+          <x:t>Tychy</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G21" t="inlineStr">
+        <x:is>
+          <x:t>śląskie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H21" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="inlineStr">
+        <x:is>
+          <x:t>03-264</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B22" t="inlineStr">
+        <x:is>
+          <x:t>Warszawa</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C22" t="inlineStr">
+        <x:is>
+          <x:t>Ojca Aniceta</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D22" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E22" t="inlineStr">
+        <x:is>
+          <x:t>Warszawa</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F22" t="inlineStr">
+        <x:is>
+          <x:t>Warszawa</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G22" t="inlineStr">
+        <x:is>
+          <x:t>mazowieckie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H22" t="inlineStr">
+        <x:is>
+          <x:t>Brak ulicy</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="inlineStr">
+        <x:is>
+          <x:t>03-264</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B23" t="inlineStr">
+        <x:is>
+          <x:t>Warszawa</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C23" t="inlineStr">
+        <x:is>
+          <x:t>Ojca Aniceta</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D23" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E23" t="inlineStr">
+        <x:is>
+          <x:t>Warszawa</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F23" t="inlineStr">
+        <x:is>
+          <x:t>Warszawa</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G23" t="inlineStr">
+        <x:is>
+          <x:t>mazowieckie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H23" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="inlineStr">
+        <x:is>
+          <x:t>50-153</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B24" t="inlineStr">
+        <x:is>
+          <x:t>Wrocław</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C24" t="inlineStr">
+        <x:is>
+          <x:t>św. Ducha</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D24" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E24" t="inlineStr">
+        <x:is>
+          <x:t>Wrocław</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F24" t="inlineStr">
+        <x:is>
+          <x:t>Wrocław</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G24" t="inlineStr">
+        <x:is>
+          <x:t>dolnośląskie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H24" t="inlineStr">
+        <x:is>
+          <x:t>Brak ulicy</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" t="inlineStr">
+        <x:is>
+          <x:t>50-153</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B25" t="inlineStr">
+        <x:is>
+          <x:t>Wrocław</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C25" t="inlineStr">
+        <x:is>
+          <x:t>św. Ducha</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D25" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E25" t="inlineStr">
+        <x:is>
+          <x:t>Wrocław</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F25" t="inlineStr">
+        <x:is>
+          <x:t>Wrocław</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G25" t="inlineStr">
+        <x:is>
+          <x:t>dolnośląskie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H25" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" t="inlineStr">
+        <x:is>
+          <x:t>65-088</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B26" t="inlineStr">
+        <x:is>
+          <x:t>Zielona Góra</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C26" t="inlineStr">
+        <x:is>
+          <x:t>Baudouina</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D26" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E26" t="inlineStr">
+        <x:is>
+          <x:t>Zielona Góra</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F26" t="inlineStr">
+        <x:is>
+          <x:t>Zielona Góra</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G26" t="inlineStr">
+        <x:is>
+          <x:t>lubuskie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H26" t="inlineStr">
+        <x:is>
+          <x:t>Brak ulicy</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="inlineStr">
+        <x:is>
+          <x:t>65-088</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B27" t="inlineStr">
+        <x:is>
+          <x:t>Zielona Góra</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C27" t="inlineStr">
+        <x:is>
+          <x:t>Baudouina</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D27" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E27" t="inlineStr">
+        <x:is>
+          <x:t>Zielona Góra</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F27" t="inlineStr">
+        <x:is>
+          <x:t>Zielona Góra</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G27" t="inlineStr">
+        <x:is>
+          <x:t>lubuskie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H27" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="inlineStr">
+        <x:is>
           <x:t>66-006</x:t>
         </x:is>
       </x:c>
-      <x:c r="B13" t="inlineStr">
+      <x:c r="B28" t="inlineStr">
         <x:is>
           <x:t>Zielona Góra</x:t>
         </x:is>
       </x:c>
-      <x:c r="C13" t="inlineStr">
+      <x:c r="C28" t="inlineStr">
         <x:is>
           <x:t>Ochla-Osiedle Dworskie</x:t>
         </x:is>
       </x:c>
-      <x:c r="D13" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E13" t="inlineStr">
+      <x:c r="D28" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E28" t="inlineStr">
         <x:is>
           <x:t>Zielona Góra</x:t>
         </x:is>
       </x:c>
-      <x:c r="F13" t="inlineStr">
+      <x:c r="F28" t="inlineStr">
         <x:is>
           <x:t>Zielona Góra</x:t>
         </x:is>
       </x:c>
-      <x:c r="G13" t="inlineStr">
+      <x:c r="G28" t="inlineStr">
         <x:is>
           <x:t>lubuskie</x:t>
         </x:is>
       </x:c>
-      <x:c r="H13" t="inlineStr">
+      <x:c r="H28" t="inlineStr">
+        <x:is>
+          <x:t>Brak ulicy</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="inlineStr">
+        <x:is>
+          <x:t>66-006</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B29" t="inlineStr">
+        <x:is>
+          <x:t>Zielona Góra</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C29" t="inlineStr">
+        <x:is>
+          <x:t>Ochla-Osiedle Dworskie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D29" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E29" t="inlineStr">
+        <x:is>
+          <x:t>Zielona Góra</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F29" t="inlineStr">
+        <x:is>
+          <x:t>Zielona Góra</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G29" t="inlineStr">
+        <x:is>
+          <x:t>lubuskie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H29" t="inlineStr">
         <x:is>
           <x:t/>
         </x:is>

</xml_diff>

<commit_message>
Wszystko działa, zostało 12 błędów przy ładowaniu kodów
</commit_message>
<xml_diff>
--- a/TerytLoad/AppData/pna/BledyPnaPropozycje.xlsx
+++ b/TerytLoad/AppData/pna/BledyPnaPropozycje.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Błędy PNA" sheetId="1" r:id="Rab979c9e76144726"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Błędy PNA" sheetId="1" r:id="Rac0aa5e259ca423c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -139,17 +139,17 @@
     <x:row r="4">
       <x:c r="A4" t="inlineStr">
         <x:is>
-          <x:t>48-300</x:t>
+          <x:t>15-568</x:t>
         </x:is>
       </x:c>
       <x:c r="B4" t="inlineStr">
         <x:is>
-          <x:t>Nysa</x:t>
+          <x:t>Białystok</x:t>
         </x:is>
       </x:c>
       <x:c r="C4" t="inlineStr">
         <x:is>
-          <x:t>Generała Augusta Emila Fieldorfa-Pseudonim Nil</x:t>
+          <x:t>św. Proroka Eliasza</x:t>
         </x:is>
       </x:c>
       <x:c r="D4" t="inlineStr">
@@ -159,17 +159,17 @@
       </x:c>
       <x:c r="E4" t="inlineStr">
         <x:is>
-          <x:t>Nysa</x:t>
+          <x:t>Białystok</x:t>
         </x:is>
       </x:c>
       <x:c r="F4" t="inlineStr">
         <x:is>
-          <x:t>nyski</x:t>
+          <x:t>Białystok</x:t>
         </x:is>
       </x:c>
       <x:c r="G4" t="inlineStr">
         <x:is>
-          <x:t>opolskie</x:t>
+          <x:t>podlaskie</x:t>
         </x:is>
       </x:c>
       <x:c r="H4" t="inlineStr">
@@ -181,17 +181,17 @@
     <x:row r="5">
       <x:c r="A5" t="inlineStr">
         <x:is>
-          <x:t>48-300</x:t>
+          <x:t>15-568</x:t>
         </x:is>
       </x:c>
       <x:c r="B5" t="inlineStr">
         <x:is>
-          <x:t>Nysa</x:t>
+          <x:t>Białystok</x:t>
         </x:is>
       </x:c>
       <x:c r="C5" t="inlineStr">
         <x:is>
-          <x:t>Generała Augusta Emila Fieldorfa-Pseudonim Nil</x:t>
+          <x:t>św. Proroka Eliasza</x:t>
         </x:is>
       </x:c>
       <x:c r="D5" t="inlineStr">
@@ -201,17 +201,17 @@
       </x:c>
       <x:c r="E5" t="inlineStr">
         <x:is>
-          <x:t>Nysa</x:t>
+          <x:t>Białystok</x:t>
         </x:is>
       </x:c>
       <x:c r="F5" t="inlineStr">
         <x:is>
-          <x:t>nyski</x:t>
+          <x:t>Białystok</x:t>
         </x:is>
       </x:c>
       <x:c r="G5" t="inlineStr">
         <x:is>
-          <x:t>opolskie</x:t>
+          <x:t>podlaskie</x:t>
         </x:is>
       </x:c>
       <x:c r="H5" t="inlineStr">
@@ -223,17 +223,17 @@
     <x:row r="6">
       <x:c r="A6" t="inlineStr">
         <x:is>
-          <x:t>42-256</x:t>
+          <x:t>85-791</x:t>
         </x:is>
       </x:c>
       <x:c r="B6" t="inlineStr">
         <x:is>
-          <x:t>Olsztyn</x:t>
+          <x:t>Bydgoszcz</x:t>
         </x:is>
       </x:c>
       <x:c r="C6" t="inlineStr">
         <x:is>
-          <x:t>Plac im. marszałka Józefa Piłsudskiego</x:t>
+          <x:t>pl. plac św. Mateusza Apostoła i Ewangelisty</x:t>
         </x:is>
       </x:c>
       <x:c r="D6" t="inlineStr">
@@ -243,17 +243,17 @@
       </x:c>
       <x:c r="E6" t="inlineStr">
         <x:is>
-          <x:t>Olsztyn</x:t>
+          <x:t>Bydgoszcz</x:t>
         </x:is>
       </x:c>
       <x:c r="F6" t="inlineStr">
         <x:is>
-          <x:t>częstochowski</x:t>
+          <x:t>Bydgoszcz</x:t>
         </x:is>
       </x:c>
       <x:c r="G6" t="inlineStr">
         <x:is>
-          <x:t>śląskie</x:t>
+          <x:t>kujawsko-pomorskie</x:t>
         </x:is>
       </x:c>
       <x:c r="H6" t="inlineStr">
@@ -265,17 +265,17 @@
     <x:row r="7">
       <x:c r="A7" t="inlineStr">
         <x:is>
-          <x:t>42-256</x:t>
+          <x:t>85-791</x:t>
         </x:is>
       </x:c>
       <x:c r="B7" t="inlineStr">
         <x:is>
-          <x:t>Olsztyn</x:t>
+          <x:t>Bydgoszcz</x:t>
         </x:is>
       </x:c>
       <x:c r="C7" t="inlineStr">
         <x:is>
-          <x:t>Plac im. marszałka Józefa Piłsudskiego</x:t>
+          <x:t>pl. plac św. Mateusza Apostoła i Ewangelisty</x:t>
         </x:is>
       </x:c>
       <x:c r="D7" t="inlineStr">
@@ -285,17 +285,17 @@
       </x:c>
       <x:c r="E7" t="inlineStr">
         <x:is>
-          <x:t>Olsztyn</x:t>
+          <x:t>Bydgoszcz</x:t>
         </x:is>
       </x:c>
       <x:c r="F7" t="inlineStr">
         <x:is>
-          <x:t>częstochowski</x:t>
+          <x:t>Bydgoszcz</x:t>
         </x:is>
       </x:c>
       <x:c r="G7" t="inlineStr">
         <x:is>
-          <x:t>śląskie</x:t>
+          <x:t>kujawsko-pomorskie</x:t>
         </x:is>
       </x:c>
       <x:c r="H7" t="inlineStr">
@@ -307,17 +307,17 @@
     <x:row r="8">
       <x:c r="A8" t="inlineStr">
         <x:is>
-          <x:t>07-310</x:t>
+          <x:t>80-893</x:t>
         </x:is>
       </x:c>
       <x:c r="B8" t="inlineStr">
         <x:is>
-          <x:t>Ostrów Mazowiecka</x:t>
+          <x:t>Gdańsk</x:t>
         </x:is>
       </x:c>
       <x:c r="C8" t="inlineStr">
         <x:is>
-          <x:t>Spokojna</x:t>
+          <x:t>Bastion św. Elżbiety</x:t>
         </x:is>
       </x:c>
       <x:c r="D8" t="inlineStr">
@@ -327,17 +327,17 @@
       </x:c>
       <x:c r="E8" t="inlineStr">
         <x:is>
-          <x:t>Ostrów Mazowiecka</x:t>
+          <x:t>Gdańsk</x:t>
         </x:is>
       </x:c>
       <x:c r="F8" t="inlineStr">
         <x:is>
-          <x:t>ostrowski</x:t>
+          <x:t>Gdańsk</x:t>
         </x:is>
       </x:c>
       <x:c r="G8" t="inlineStr">
         <x:is>
-          <x:t>mazowieckie</x:t>
+          <x:t>pomorskie</x:t>
         </x:is>
       </x:c>
       <x:c r="H8" t="inlineStr">
@@ -349,17 +349,17 @@
     <x:row r="9">
       <x:c r="A9" t="inlineStr">
         <x:is>
-          <x:t>07-310</x:t>
+          <x:t>80-893</x:t>
         </x:is>
       </x:c>
       <x:c r="B9" t="inlineStr">
         <x:is>
-          <x:t>Ostrów Mazowiecka</x:t>
+          <x:t>Gdańsk</x:t>
         </x:is>
       </x:c>
       <x:c r="C9" t="inlineStr">
         <x:is>
-          <x:t>Spokojna</x:t>
+          <x:t>Bastion św. Elżbiety</x:t>
         </x:is>
       </x:c>
       <x:c r="D9" t="inlineStr">
@@ -369,17 +369,17 @@
       </x:c>
       <x:c r="E9" t="inlineStr">
         <x:is>
-          <x:t>Ostrów Mazowiecka</x:t>
+          <x:t>Gdańsk</x:t>
         </x:is>
       </x:c>
       <x:c r="F9" t="inlineStr">
         <x:is>
-          <x:t>ostrowski</x:t>
+          <x:t>Gdańsk</x:t>
         </x:is>
       </x:c>
       <x:c r="G9" t="inlineStr">
         <x:is>
-          <x:t>mazowieckie</x:t>
+          <x:t>pomorskie</x:t>
         </x:is>
       </x:c>
       <x:c r="H9" t="inlineStr">
@@ -391,17 +391,17 @@
     <x:row r="10">
       <x:c r="A10" t="inlineStr">
         <x:is>
-          <x:t>71-602</x:t>
+          <x:t>81-402</x:t>
         </x:is>
       </x:c>
       <x:c r="B10" t="inlineStr">
         <x:is>
-          <x:t>Szczecin</x:t>
+          <x:t>Gdynia</x:t>
         </x:is>
       </x:c>
       <x:c r="C10" t="inlineStr">
         <x:is>
-          <x:t>Storrady-Świętosławy</x:t>
+          <x:t>bp. Dominika</x:t>
         </x:is>
       </x:c>
       <x:c r="D10" t="inlineStr">
@@ -411,17 +411,17 @@
       </x:c>
       <x:c r="E10" t="inlineStr">
         <x:is>
-          <x:t>Szczecin</x:t>
+          <x:t>Gdynia</x:t>
         </x:is>
       </x:c>
       <x:c r="F10" t="inlineStr">
         <x:is>
-          <x:t>Szczecin</x:t>
+          <x:t>Gdynia</x:t>
         </x:is>
       </x:c>
       <x:c r="G10" t="inlineStr">
         <x:is>
-          <x:t>zachodniopomorskie</x:t>
+          <x:t>pomorskie</x:t>
         </x:is>
       </x:c>
       <x:c r="H10" t="inlineStr">
@@ -433,40 +433,628 @@
     <x:row r="11">
       <x:c r="A11" t="inlineStr">
         <x:is>
+          <x:t>81-402</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B11" t="inlineStr">
+        <x:is>
+          <x:t>Gdynia</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C11" t="inlineStr">
+        <x:is>
+          <x:t>bp. Dominika</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D11" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E11" t="inlineStr">
+        <x:is>
+          <x:t>Gdynia</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F11" t="inlineStr">
+        <x:is>
+          <x:t>Gdynia</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G11" t="inlineStr">
+        <x:is>
+          <x:t>pomorskie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H11" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="inlineStr">
+        <x:is>
+          <x:t>48-300</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B12" t="inlineStr">
+        <x:is>
+          <x:t>Nysa</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C12" t="inlineStr">
+        <x:is>
+          <x:t>Generała Augusta Emila Fieldorfa-Pseudonim Nil</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D12" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E12" t="inlineStr">
+        <x:is>
+          <x:t>Nysa</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F12" t="inlineStr">
+        <x:is>
+          <x:t>nyski</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G12" t="inlineStr">
+        <x:is>
+          <x:t>opolskie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H12" t="inlineStr">
+        <x:is>
+          <x:t>Brak ulicy</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="inlineStr">
+        <x:is>
+          <x:t>48-300</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B13" t="inlineStr">
+        <x:is>
+          <x:t>Nysa</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C13" t="inlineStr">
+        <x:is>
+          <x:t>Generała Augusta Emila Fieldorfa-Pseudonim Nil</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D13" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E13" t="inlineStr">
+        <x:is>
+          <x:t>Nysa</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F13" t="inlineStr">
+        <x:is>
+          <x:t>nyski</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G13" t="inlineStr">
+        <x:is>
+          <x:t>opolskie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H13" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="inlineStr">
+        <x:is>
+          <x:t>42-256</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B14" t="inlineStr">
+        <x:is>
+          <x:t>Olsztyn</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C14" t="inlineStr">
+        <x:is>
+          <x:t>Plac im. marszałka Józefa Piłsudskiego</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D14" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E14" t="inlineStr">
+        <x:is>
+          <x:t>Olsztyn</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F14" t="inlineStr">
+        <x:is>
+          <x:t>częstochowski</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G14" t="inlineStr">
+        <x:is>
+          <x:t>śląskie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H14" t="inlineStr">
+        <x:is>
+          <x:t>Brak ulicy</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="inlineStr">
+        <x:is>
+          <x:t>42-256</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B15" t="inlineStr">
+        <x:is>
+          <x:t>Olsztyn</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C15" t="inlineStr">
+        <x:is>
+          <x:t>Plac im. marszałka Józefa Piłsudskiego</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D15" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E15" t="inlineStr">
+        <x:is>
+          <x:t>Olsztyn</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F15" t="inlineStr">
+        <x:is>
+          <x:t>częstochowski</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G15" t="inlineStr">
+        <x:is>
+          <x:t>śląskie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H15" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="inlineStr">
+        <x:is>
+          <x:t>07-310</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B16" t="inlineStr">
+        <x:is>
+          <x:t>Ostrów Mazowiecka</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C16" t="inlineStr">
+        <x:is>
+          <x:t>Spokojna</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D16" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E16" t="inlineStr">
+        <x:is>
+          <x:t>Ostrów Mazowiecka</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F16" t="inlineStr">
+        <x:is>
+          <x:t>ostrowski</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G16" t="inlineStr">
+        <x:is>
+          <x:t>mazowieckie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H16" t="inlineStr">
+        <x:is>
+          <x:t>Brak ulicy</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="inlineStr">
+        <x:is>
+          <x:t>07-310</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B17" t="inlineStr">
+        <x:is>
+          <x:t>Ostrów Mazowiecka</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C17" t="inlineStr">
+        <x:is>
+          <x:t>Spokojna</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D17" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E17" t="inlineStr">
+        <x:is>
+          <x:t>Ostrów Mazowiecka</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F17" t="inlineStr">
+        <x:is>
+          <x:t>ostrowski</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G17" t="inlineStr">
+        <x:is>
+          <x:t>mazowieckie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H17" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="inlineStr">
+        <x:is>
+          <x:t>41-711</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B18" t="inlineStr">
+        <x:is>
+          <x:t>Ruda Śląska</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C18" t="inlineStr">
+        <x:is>
+          <x:t>Dr. Jordana</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D18" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E18" t="inlineStr">
+        <x:is>
+          <x:t>Ruda Śląska</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F18" t="inlineStr">
+        <x:is>
+          <x:t>Ruda Śląska</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G18" t="inlineStr">
+        <x:is>
+          <x:t>śląskie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H18" t="inlineStr">
+        <x:is>
+          <x:t>Brak ulicy</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="inlineStr">
+        <x:is>
+          <x:t>41-711</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B19" t="inlineStr">
+        <x:is>
+          <x:t>Ruda Śląska</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C19" t="inlineStr">
+        <x:is>
+          <x:t>Dr. Jordana</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D19" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E19" t="inlineStr">
+        <x:is>
+          <x:t>Ruda Śląska</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F19" t="inlineStr">
+        <x:is>
+          <x:t>Ruda Śląska</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G19" t="inlineStr">
+        <x:is>
+          <x:t>śląskie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H19" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="inlineStr">
+        <x:is>
           <x:t>71-602</x:t>
         </x:is>
       </x:c>
-      <x:c r="B11" t="inlineStr">
+      <x:c r="B20" t="inlineStr">
         <x:is>
           <x:t>Szczecin</x:t>
         </x:is>
       </x:c>
-      <x:c r="C11" t="inlineStr">
+      <x:c r="C20" t="inlineStr">
         <x:is>
           <x:t>Storrady-Świętosławy</x:t>
         </x:is>
       </x:c>
-      <x:c r="D11" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c r="E11" t="inlineStr">
+      <x:c r="D20" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E20" t="inlineStr">
         <x:is>
           <x:t>Szczecin</x:t>
         </x:is>
       </x:c>
-      <x:c r="F11" t="inlineStr">
+      <x:c r="F20" t="inlineStr">
         <x:is>
           <x:t>Szczecin</x:t>
         </x:is>
       </x:c>
-      <x:c r="G11" t="inlineStr">
+      <x:c r="G20" t="inlineStr">
         <x:is>
           <x:t>zachodniopomorskie</x:t>
         </x:is>
       </x:c>
-      <x:c r="H11" t="inlineStr">
+      <x:c r="H20" t="inlineStr">
+        <x:is>
+          <x:t>Brak ulicy</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="inlineStr">
+        <x:is>
+          <x:t>71-602</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B21" t="inlineStr">
+        <x:is>
+          <x:t>Szczecin</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C21" t="inlineStr">
+        <x:is>
+          <x:t>Storrady-Świętosławy</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D21" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E21" t="inlineStr">
+        <x:is>
+          <x:t>Szczecin</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F21" t="inlineStr">
+        <x:is>
+          <x:t>Szczecin</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G21" t="inlineStr">
+        <x:is>
+          <x:t>zachodniopomorskie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H21" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="inlineStr">
+        <x:is>
+          <x:t>02-647</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B22" t="inlineStr">
+        <x:is>
+          <x:t>Warszawa</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C22" t="inlineStr">
+        <x:is>
+          <x:t>Rabindranatha Tagore</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D22" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E22" t="inlineStr">
+        <x:is>
+          <x:t>Warszawa</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F22" t="inlineStr">
+        <x:is>
+          <x:t>Warszawa</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G22" t="inlineStr">
+        <x:is>
+          <x:t>mazowieckie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H22" t="inlineStr">
+        <x:is>
+          <x:t>Brak ulicy</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="inlineStr">
+        <x:is>
+          <x:t>02-647</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B23" t="inlineStr">
+        <x:is>
+          <x:t>Warszawa</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C23" t="inlineStr">
+        <x:is>
+          <x:t>Rabindranatha Tagore</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D23" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E23" t="inlineStr">
+        <x:is>
+          <x:t>Warszawa</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F23" t="inlineStr">
+        <x:is>
+          <x:t>Warszawa</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G23" t="inlineStr">
+        <x:is>
+          <x:t>mazowieckie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H23" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="inlineStr">
+        <x:is>
+          <x:t>41-800</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B24" t="inlineStr">
+        <x:is>
+          <x:t>Zabrze</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C24" t="inlineStr">
+        <x:is>
+          <x:t>Góry św. Anny</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D24" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E24" t="inlineStr">
+        <x:is>
+          <x:t>Zabrze</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F24" t="inlineStr">
+        <x:is>
+          <x:t>Zabrze</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G24" t="inlineStr">
+        <x:is>
+          <x:t>śląskie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H24" t="inlineStr">
+        <x:is>
+          <x:t>Brak ulicy</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" t="inlineStr">
+        <x:is>
+          <x:t>41-800</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B25" t="inlineStr">
+        <x:is>
+          <x:t>Zabrze</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C25" t="inlineStr">
+        <x:is>
+          <x:t>Góry św. Anny</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D25" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E25" t="inlineStr">
+        <x:is>
+          <x:t>Zabrze</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F25" t="inlineStr">
+        <x:is>
+          <x:t>Zabrze</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G25" t="inlineStr">
+        <x:is>
+          <x:t>śląskie</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H25" t="inlineStr">
         <x:is>
           <x:t/>
         </x:is>

</xml_diff>